<commit_message>
Add CTL/TSS baseline targets to Oversigt
</commit_message>
<xml_diff>
--- a/data/Master_Plan.xlsx
+++ b/data/Master_Plan.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:U15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -503,6 +503,11 @@
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="26" customWidth="1" min="15" max="15"/>
     <col width="45" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -586,6 +591,31 @@
           <t>Note</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Target CTL (start)</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Target CTL (slut)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Target TSS</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Afvigelse (Faktisk-Target TSS)</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>TSB-mål / note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -646,6 +676,23 @@
       <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Uge gennemført. 4 løb var for mange — fra uge 2 max 3/uge.</t>
+        </is>
+      </c>
+      <c r="Q2" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="R2" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="S2" s="6" t="n">
+        <v>290</v>
+      </c>
+      <c r="T2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" s="6" t="inlineStr">
+        <is>
+          <t>Etableringsuge — TSB endte -8</t>
         </is>
       </c>
     </row>
@@ -698,6 +745,21 @@
       <c r="P3" s="2" t="inlineStr">
         <is>
           <t>2 VO2-stimuli (tirs løb + lør cykel-bjerg). Cykel-volumen på Mallorca.</t>
+        </is>
+      </c>
+      <c r="Q3" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="R3" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="S3" s="6" t="n">
+        <v>340</v>
+      </c>
+      <c r="T3" s="6" t="n"/>
+      <c r="U3" s="6" t="inlineStr">
+        <is>
+          <t>TSB ca. -10 til -15</t>
         </is>
       </c>
     </row>
@@ -748,6 +810,21 @@
           <t>Mallorca-camp. Lang løb/svøm man, lang cykel tirs, VO2 cykel ons, hjemflyvning tors, styrke fre, løb 60 min lør, svøm søn. TSB ~-36.</t>
         </is>
       </c>
+      <c r="Q4" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="R4" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="S4" s="6" t="n">
+        <v>370</v>
+      </c>
+      <c r="T4" s="6" t="n"/>
+      <c r="U4" s="6" t="inlineStr">
+        <is>
+          <t>Camp-uge — TSB max -35/-36 ok</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -796,6 +873,21 @@
           <t>Restitutionsuge efter 3 build-uger. Lavere volumen, ingen Z4/Z5.</t>
         </is>
       </c>
+      <c r="Q5" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="T5" s="6" t="n"/>
+      <c r="U5" s="6" t="inlineStr">
+        <is>
+          <t>TSB stiger mod -5 til 0</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -844,6 +936,21 @@
           <t>Tilbage til hverdagsrytme.</t>
         </is>
       </c>
+      <c r="Q6" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="R6" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="S6" s="6" t="n">
+        <v>385</v>
+      </c>
+      <c r="T6" s="6" t="n"/>
+      <c r="U6" s="6" t="inlineStr">
+        <is>
+          <t>TSB ca. -10 til -15</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -892,6 +999,21 @@
           <t>Rejseuge — let cykel/løb, vedligehold.</t>
         </is>
       </c>
+      <c r="Q7" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>320</v>
+      </c>
+      <c r="T7" s="6" t="n"/>
+      <c r="U7" s="6" t="inlineStr">
+        <is>
+          <t>Rejseuge — lavere belastning</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -940,6 +1062,21 @@
           <t>Stor cykel-uge #2.</t>
         </is>
       </c>
+      <c r="Q8" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="R8" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="S8" s="6" t="n">
+        <v>430</v>
+      </c>
+      <c r="T8" s="6" t="n"/>
+      <c r="U8" s="6" t="inlineStr">
+        <is>
+          <t>Camp-uge — TSB kan nå -30/-35</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -988,6 +1125,21 @@
           <t>Restitution + rejsedag hjem.</t>
         </is>
       </c>
+      <c r="Q9" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="S9" s="6" t="n">
+        <v>215</v>
+      </c>
+      <c r="T9" s="6" t="n"/>
+      <c r="U9" s="6" t="inlineStr">
+        <is>
+          <t>TSB stiger mod 0</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1036,6 +1188,21 @@
           <t>Musik i Gentofte i ugen efter (31/7–2/8) – planlæg let.</t>
         </is>
       </c>
+      <c r="Q10" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="R10" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="S10" s="6" t="n">
+        <v>440</v>
+      </c>
+      <c r="T10" s="6" t="n"/>
+      <c r="U10" s="6" t="inlineStr">
+        <is>
+          <t>TSB ca. -10 til -15</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1084,6 +1251,21 @@
           <t>Svømme-fokus øges mod Christiansborg Rundt.</t>
         </is>
       </c>
+      <c r="Q11" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>470</v>
+      </c>
+      <c r="T11" s="6" t="n"/>
+      <c r="U11" s="6" t="inlineStr">
+        <is>
+          <t>TSB ca. -15</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1132,6 +1314,21 @@
           <t>Sidste store blok før pre-race.</t>
         </is>
       </c>
+      <c r="Q12" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="R12" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="S12" s="6" t="n">
+        <v>470</v>
+      </c>
+      <c r="T12" s="6" t="n"/>
+      <c r="U12" s="6" t="inlineStr">
+        <is>
+          <t>Peak CTL — sidste hårde blok</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -1180,6 +1377,21 @@
           <t>Svømme-specifik uge, nedtrapning starter. Norway 22–24/8 – planlæg rejse.</t>
         </is>
       </c>
+      <c r="Q13" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="R13" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="S13" s="6" t="n">
+        <v>275</v>
+      </c>
+      <c r="T13" s="6" t="n"/>
+      <c r="U13" s="6" t="inlineStr">
+        <is>
+          <t>Taper start — TSB stiger mod +5</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -1228,6 +1440,21 @@
           <t>Race week: 2000 m svøm 29/8. Taper ind, kort løb.</t>
         </is>
       </c>
+      <c r="Q14" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="R14" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="S14" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="T14" s="6" t="n"/>
+      <c r="U14" s="6" t="inlineStr">
+        <is>
+          <t>Christiansborg 29/8 — TSB target +5 til +10</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
@@ -1274,6 +1501,21 @@
       <c r="P15" s="5" t="inlineStr">
         <is>
           <t>Marathon Médoc 5/9. Efter race: planen forlænges med recovery/2027-base – udfyldes når vi når hertil.</t>
+        </is>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="T15" s="6" t="n"/>
+      <c r="U15" s="6" t="inlineStr">
+        <is>
+          <t>Marathon Médoc 5/9 — TSB target +10 til +15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update: masterplan uge 3 justeret — løb man, cykel tirs, svøm ons
</commit_message>
<xml_diff>
--- a/data/Master_Plan.xlsx
+++ b/data/Master_Plan.xlsx
@@ -2366,17 +2366,17 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Svøm+Løb</t>
+          <t>Løb</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Svøm + lang løb</t>
+          <t>Lang løb Z2</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>30+60 min</t>
+          <t>90 min</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -2385,11 +2385,11 @@
         </is>
       </c>
       <c r="I16" s="6" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>Møde kl. 13:00 — træning afsluttet inden. Lang løb Z2 base.</t>
+          <t>Lang løb Z2 base. Ingen svøm denne dag — svøm flyttet til onsdag.</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
@@ -2424,12 +2424,12 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Lang cykel + open-water svøm</t>
+          <t>Cykel Formentor 149km</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>2,5-3 t + 20 min</t>
+          <t>5-6 t</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -2438,11 +2438,11 @@
         </is>
       </c>
       <c r="I17" s="6" t="n">
-        <v>130</v>
+        <v>160</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>Mallorca volumen-dag. Ekstra open-water svøm til Christiansborg.</t>
+          <t>Mallorca volumen-dag. Formentor-ruten. Open-water svøm udgår (svøm på onsdag).</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
@@ -2472,30 +2472,30 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Cykel</t>
+          <t>Svøm</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>VO2 cykel-intervaller</t>
+          <t>Svøm 1500m let teknisk</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>75 min</t>
+          <t>45 min</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>Z4-Z5</t>
+          <t>Z1-Z2</t>
         </is>
       </c>
       <c r="I18" s="6" t="n">
-        <v>75</v>
+        <v>35</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>VO2-stimulus #1 i uge 3. Strukturerede intervaller.</t>
+          <t>Teknisk svøm — VO2 cykel-intervaller erstattet med svøm denne uge.</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Uge 3 faktiske tal (TSS 386, CTL 40→43, TSB -12, AF 7/7) + uge 4 restitutionsplan aftalt med Kennet
</commit_message>
<xml_diff>
--- a/data/Master_Plan.xlsx
+++ b/data/Master_Plan.xlsx
@@ -782,32 +782,46 @@
           <t>Mallorca</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
+      <c r="E4" s="2" t="n">
+        <v>370</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>386</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>-12</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>21.7</v>
+      </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>?/7</t>
+          <t>7/7</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>OK – løb reduceret 75→60 min (TSB-floor)</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>Mallorca-camp. Lang løb/svøm man, lang cykel tirs, VO2 cykel ons, hjemflyvning tors, styrke fre, løb 60 min lør, svøm søn. TSB ~-36.</t>
+          <t>Mallorca-camp gennemført. Formentor 149km (7,5t, TSS 128) tirsdag — ugens nøglepas. Løb reduceret til 60 min lørdag som planlagt (TSB-floor). Søndag byttet svøm til langcykel (173 min) hjemme. TSB-lavpunkt -26 i ugen, endte -12 ved ugeskifte — bedre end ventet. Alle Friel-regler overholdt (TSB &gt; -35-loft, max 3 løb/uge, recovery-uge planlagt efter).</t>
         </is>
       </c>
       <c r="Q4" s="6" t="n">
@@ -819,7 +833,9 @@
       <c r="S4" s="6" t="n">
         <v>370</v>
       </c>
-      <c r="T4" s="6" t="n"/>
+      <c r="T4" s="6" t="n">
+        <v>16</v>
+      </c>
       <c r="U4" s="6" t="inlineStr">
         <is>
           <t>Camp-uge — TSB max -35/-36 ok</t>
@@ -845,9 +861,13 @@
           <t>Gentofte</t>
         </is>
       </c>
-      <c r="E5" s="3" t="n"/>
+      <c r="E5" s="3" t="n">
+        <v>195</v>
+      </c>
       <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
+      <c r="G5" s="3" t="n">
+        <v>43</v>
+      </c>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
@@ -865,12 +885,12 @@
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>Restitutionsuge efter 3 build-uger. Lavere volumen, ingen Z4/Z5.</t>
+          <t>Restitutionsuge tilpasset DK-hverdag: let svøm man (før hjemmekontor), løb tirs (god formiddag), kort spin ons (workshop-dag), cykel tor kl. 16 (job fylder formiddag), hvile fre (Ædge Dag), langt løb 1,5t lør (udvidet efter ønske), let svøm søn. Ingen Z4/Z5, 0 VO2-stimuli, 2 løb. TSS 195 er lidt over oprindeligt mål (180) pga. forlænget lørdagsløb — stadig restitutionsniveau.</t>
         </is>
       </c>
       <c r="Q5" s="6" t="n">
@@ -2376,7 +2396,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>90 min</t>
+          <t>89 min</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -2385,16 +2405,16 @@
         </is>
       </c>
       <c r="I16" s="6" t="n">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>Lang løb Z2 base. Ingen svøm denne dag — svøm flyttet til onsdag.</t>
+          <t>Sóller. Som planlagt — formiddag før møde kl 13.</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Planlagt</t>
+          <t>Udført</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2439,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Cykel+Svøm</t>
+          <t>Cykel</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -2429,7 +2449,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>5-6 t</t>
+          <t>7,5 t</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -2438,16 +2458,16 @@
         </is>
       </c>
       <c r="I17" s="6" t="n">
-        <v>160</v>
+        <v>128</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>Mallorca volumen-dag. Formentor-ruten. Open-water svøm udgår (svøm på onsdag).</t>
+          <t>Fornalutx. Længere end estimeret (448 min vs 5-6t), men lavere TSS end ventet — overvejende Z2.</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>Planlagt</t>
+          <t>Udført</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2487,7 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -2477,12 +2497,12 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Svøm 1500m let teknisk</t>
+          <t>Open water svøm let</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>45 min</t>
+          <t>34 min</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -2491,16 +2511,16 @@
         </is>
       </c>
       <c r="I18" s="6" t="n">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>Teknisk svøm — VO2 cykel-intervaller erstattet med svøm denne uge.</t>
+          <t>Sóller. Som planlagt.</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>Planlagt</t>
+          <t>Udført</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2540,7 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -2535,7 +2555,7 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>60 min</t>
+          <t>95 min</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -2544,16 +2564,16 @@
         </is>
       </c>
       <c r="I19" s="6" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>Sidste dag i Mallorca — fly hjem aften. Let spin.</t>
+          <t>Fornalutx → fly hjem aften. Lidt længere end planlagt 60 min.</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>Planlagt</t>
+          <t>Udført</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2593,7 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>07:25</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -2583,12 +2603,12 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Styrke fuld</t>
+          <t>Styrke</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>45 min</t>
+          <t>30 min</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -2597,16 +2617,16 @@
         </is>
       </c>
       <c r="I20" s="6" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>Hjemme igen. Fuldt styrkeprogram.</t>
+          <t>Hjemme efter hjemrejse. Kortere end planlagt 45 min.</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Planlagt</t>
+          <t>Udført</t>
         </is>
       </c>
     </row>
@@ -2626,22 +2646,22 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>08:59</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Løb</t>
+          <t>Løb+Cykel</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Løb</t>
+          <t>Løb + ekstra let cykel</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>60 min</t>
+          <t>60+42 min</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -2650,16 +2670,16 @@
         </is>
       </c>
       <c r="I21" s="6" t="n">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>Reduceret fra 75→60 min efter Friel TSB-analyse (TSB endte ~-36).</t>
+          <t>Løb som planlagt 60 min (TSB-floor). Plus uplanlagt let cykeltur 42 min samme dag.</t>
         </is>
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>Planlagt</t>
+          <t>Udført</t>
         </is>
       </c>
     </row>
@@ -2679,40 +2699,40 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>09:31</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Svøm</t>
+          <t>Cykel</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Svøm</t>
+          <t>Cykel (byttet fra svøm)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>45 min</t>
+          <t>173 min</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>Z1-Z2</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="I22" s="6" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>Afslutning på Mallorca-uge. Recovery.</t>
+          <t>Byttede planlagt svøm til lang cykeltur — Kennets eget valg på dagen.</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>Planlagt</t>
+          <t>Udført</t>
         </is>
       </c>
     </row>
@@ -2725,17 +2745,47 @@
           <t>Man</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr"/>
-      <c r="D23" s="7" t="inlineStr"/>
-      <c r="E23" s="7" t="inlineStr"/>
-      <c r="F23" s="7" t="inlineStr"/>
-      <c r="G23" s="7" t="inlineStr"/>
-      <c r="H23" s="7" t="inlineStr"/>
-      <c r="I23" s="7" t="n"/>
-      <c r="J23" s="7" t="inlineStr"/>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>22-06</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Svøm</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Svøm let recovery</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>30 min</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Z1-Z2</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>Svømmehal. Før hjemmekontor. Teknik-fokus, lav puls.</t>
+        </is>
+      </c>
       <c r="K23" s="7" t="inlineStr">
         <is>
-          <t>Ikke planlagt</t>
+          <t>Planlagt</t>
         </is>
       </c>
     </row>
@@ -2748,17 +2798,47 @@
           <t>Tirs</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr"/>
-      <c r="D24" s="7" t="inlineStr"/>
-      <c r="E24" s="7" t="inlineStr"/>
-      <c r="F24" s="7" t="inlineStr"/>
-      <c r="G24" s="7" t="inlineStr"/>
-      <c r="H24" s="7" t="inlineStr"/>
-      <c r="I24" s="7" t="n"/>
-      <c r="J24" s="7" t="inlineStr"/>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>23-06</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Løb</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Løb Z2</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>45 min</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Z2</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="J24" s="7" t="inlineStr">
+        <is>
+          <t>God formiddag — prioriteret træningsvindue.</t>
+        </is>
+      </c>
       <c r="K24" s="7" t="inlineStr">
         <is>
-          <t>Ikke planlagt</t>
+          <t>Planlagt</t>
         </is>
       </c>
     </row>
@@ -2771,17 +2851,47 @@
           <t>Ons</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
-      <c r="D25" s="7" t="inlineStr"/>
-      <c r="E25" s="7" t="inlineStr"/>
-      <c r="F25" s="7" t="inlineStr"/>
-      <c r="G25" s="7" t="inlineStr"/>
-      <c r="H25" s="7" t="inlineStr"/>
-      <c r="I25" s="7" t="n"/>
-      <c r="J25" s="7" t="inlineStr"/>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>24-06</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Cykel</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Let cykel-spin</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>30 min</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Z1-Z2</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>Workshop-dag (Ambu Marketing). Kort pas tidlig morgen.</t>
+        </is>
+      </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
-          <t>Ikke planlagt</t>
+          <t>Planlagt</t>
         </is>
       </c>
     </row>
@@ -2794,17 +2904,47 @@
           <t>Tor</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr"/>
-      <c r="D26" s="7" t="inlineStr"/>
-      <c r="E26" s="7" t="inlineStr"/>
-      <c r="F26" s="7" t="inlineStr"/>
-      <c r="G26" s="7" t="inlineStr"/>
-      <c r="H26" s="7" t="inlineStr"/>
-      <c r="I26" s="7" t="n"/>
-      <c r="J26" s="7" t="inlineStr"/>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>25-06</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Cykel</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Cykel Z2</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>45 min</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Z2</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="J26" s="7" t="inlineStr">
+        <is>
+          <t>Eftermiddag — job fylder formiddagen (Partner Platform-møde kl 11).</t>
+        </is>
+      </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>Ikke planlagt</t>
+          <t>Planlagt</t>
         </is>
       </c>
     </row>
@@ -2817,17 +2957,47 @@
           <t>Fre</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr"/>
-      <c r="D27" s="7" t="inlineStr"/>
-      <c r="E27" s="7" t="inlineStr"/>
-      <c r="F27" s="7" t="inlineStr"/>
-      <c r="G27" s="7" t="inlineStr"/>
-      <c r="H27" s="7" t="inlineStr"/>
-      <c r="I27" s="7" t="n"/>
-      <c r="J27" s="7" t="inlineStr"/>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>26-06</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Hvile</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>Ædge Dag (07-14:30) — job-fyldt. Ingen træning.</t>
+        </is>
+      </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>Ikke planlagt</t>
+          <t>Planlagt</t>
         </is>
       </c>
     </row>
@@ -2840,17 +3010,47 @@
           <t>Lør</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr"/>
-      <c r="D28" s="7" t="inlineStr"/>
-      <c r="E28" s="7" t="inlineStr"/>
-      <c r="F28" s="7" t="inlineStr"/>
-      <c r="G28" s="7" t="inlineStr"/>
-      <c r="H28" s="7" t="inlineStr"/>
-      <c r="I28" s="7" t="n"/>
-      <c r="J28" s="7" t="inlineStr"/>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>27-06</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Løb</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>Lang løb Z2</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>90 min</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Z2</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>76</v>
+      </c>
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t>God weekend — forlænget fra 45 til 90 min efter ønske.</t>
+        </is>
+      </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
-          <t>Ikke planlagt</t>
+          <t>Planlagt</t>
         </is>
       </c>
     </row>
@@ -2863,17 +3063,47 @@
           <t>Søn</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr"/>
-      <c r="D29" s="7" t="inlineStr"/>
-      <c r="E29" s="7" t="inlineStr"/>
-      <c r="F29" s="7" t="inlineStr"/>
-      <c r="G29" s="7" t="inlineStr"/>
-      <c r="H29" s="7" t="inlineStr"/>
-      <c r="I29" s="7" t="n"/>
-      <c r="J29" s="7" t="inlineStr"/>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>28-06</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Svøm</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Svøm let teknisk</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>45 min</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Z1-Z2</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>Afslutning på restitutionsugen.</t>
+        </is>
+      </c>
       <c r="K29" s="7" t="inlineStr">
         <is>
-          <t>Ikke planlagt</t>
+          <t>Planlagt</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master_Plan: opdater uge 2 og uge 4 (uge 26 check-in)
</commit_message>
<xml_diff>
--- a/data/Master_Plan.xlsx
+++ b/data/Master_Plan.xlsx
@@ -718,17 +718,27 @@
       <c r="E3" s="2" t="n">
         <v>340</v>
       </c>
-      <c r="F3" s="2" t="n"/>
+      <c r="F3" s="2" t="n">
+        <v>340</v>
+      </c>
       <c r="G3" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="n"/>
+      <c r="H3" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>-18</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>22.4</v>
+      </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>?/7</t>
+          <t>7/7</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
@@ -739,12 +749,12 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Udført</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2 VO2-stimuli (tirs løb + lør cykel-bjerg). Cykel-volumen på Mallorca.</t>
+          <t>Mallorca uge. TSS synkroniseringsfejl — alle aktiviteter viser 0. Bruger planlagt TSS.</t>
         </is>
       </c>
       <c r="Q3" s="6" t="n">
@@ -864,17 +874,27 @@
       <c r="E5" s="3" t="n">
         <v>195</v>
       </c>
-      <c r="F5" s="3" t="n"/>
+      <c r="F5" s="3" t="n">
+        <v>195</v>
+      </c>
       <c r="G5" s="3" t="n">
         <v>43</v>
       </c>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
+      <c r="H5" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>-16</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>22.2</v>
+      </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>?/7</t>
+          <t>7/7</t>
         </is>
       </c>
       <c r="M5" s="3" t="n">
@@ -885,12 +905,12 @@
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Udført</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>Restitutionsuge tilpasset DK-hverdag: let svøm man (før hjemmekontor), løb tirs (god formiddag), kort spin ons (workshop-dag), cykel tor kl. 16 (job fylder formiddag), hvile fre (Ædge Dag), langt løb 1,5t lør (udvidet efter ønske), let svøm søn. Ingen Z4/Z5, 0 VO2-stimuli, 2 løb. TSS 195 er lidt over oprindeligt mål (180) pga. forlænget lørdagsløb — stadig restitutionsniveau.</t>
+          <t>Recovery uge. Fuldt AF 7/7. Kost på sporet. Fortuvet lilletå — holdes øje med. Energi blandet sidst på ugen — normal recovery-respons.</t>
         </is>
       </c>
       <c r="Q5" s="6" t="n">

</xml_diff>

<commit_message>
feat: Master_Plan.xlsx — rekalibreret CTL-kurve + vægtmål 70 kg
</commit_message>
<xml_diff>
--- a/data/Master_Plan.xlsx
+++ b/data/Master_Plan.xlsx
@@ -977,10 +977,10 @@
         </is>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="S6" s="6" t="n">
         <v>385</v>
@@ -1040,10 +1040,10 @@
         </is>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>320</v>
@@ -1051,7 +1051,7 @@
       <c r="T7" s="6" t="n"/>
       <c r="U7" s="6" t="inlineStr">
         <is>
-          <t>Rejseuge — lavere belastning</t>
+          <t>Rejseuge Wales — lavere belastning</t>
         </is>
       </c>
     </row>
@@ -1103,18 +1103,18 @@
         </is>
       </c>
       <c r="Q8" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="R8" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="R8" s="6" t="n">
-        <v>54</v>
-      </c>
       <c r="S8" s="6" t="n">
-        <v>430</v>
+        <v>215</v>
       </c>
       <c r="T8" s="6" t="n"/>
       <c r="U8" s="6" t="inlineStr">
         <is>
-          <t>Camp-uge — TSB kan nå -30/-35</t>
+          <t>TSB stiger mod 0</t>
         </is>
       </c>
     </row>
@@ -1166,18 +1166,18 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="R9" s="6" t="n">
         <v>54</v>
       </c>
-      <c r="R9" s="6" t="n">
-        <v>50</v>
-      </c>
       <c r="S9" s="6" t="n">
-        <v>215</v>
+        <v>430</v>
       </c>
       <c r="T9" s="6" t="n"/>
       <c r="U9" s="6" t="inlineStr">
         <is>
-          <t>TSB stiger mod 0</t>
+          <t>TSB ca. -10 til -15</t>
         </is>
       </c>
     </row>
@@ -1229,18 +1229,18 @@
         </is>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="S10" s="6" t="n">
-        <v>440</v>
+        <v>380</v>
       </c>
       <c r="T10" s="6" t="n"/>
       <c r="U10" s="6" t="inlineStr">
         <is>
-          <t>TSB ca. -10 til -15</t>
+          <t>Musik i Gentofte fre-søn — reduceret</t>
         </is>
       </c>
     </row>
@@ -1292,10 +1292,10 @@
         </is>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>470</v>
@@ -1355,18 +1355,18 @@
         </is>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="S12" s="6" t="n">
-        <v>470</v>
+        <v>500</v>
       </c>
       <c r="T12" s="6" t="n"/>
       <c r="U12" s="6" t="inlineStr">
         <is>
-          <t>Peak CTL — sidste hårde blok</t>
+          <t>Peak CTL 68 — sidste hårde blok</t>
         </is>
       </c>
     </row>
@@ -1418,10 +1418,10 @@
         </is>
       </c>
       <c r="Q13" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="R13" s="6" t="n">
         <v>64</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>60</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>275</v>
@@ -1429,7 +1429,7 @@
       <c r="T13" s="6" t="n"/>
       <c r="U13" s="6" t="inlineStr">
         <is>
-          <t>Taper start — TSB stiger mod +5</t>
+          <t>Taper start — TSB stiger mod +5 (Norge 22-23/8)</t>
         </is>
       </c>
     </row>
@@ -1481,10 +1481,10 @@
         </is>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="S14" s="6" t="n">
         <v>250</v>
@@ -1544,10 +1544,10 @@
         </is>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="S15" s="6" t="n">
         <v>200</v>

</xml_diff>

<commit_message>
Goal Engine: plan.json som eneste kilde + omlagt uge 6-14 (Wales løbefokus, Mallorca 16-22/7 + 9-16/8, recovery+retest uge 9, marathon-ladder, OW-svøm)
</commit_message>
<xml_diff>
--- a/data/Master_Plan.xlsx
+++ b/data/Master_Plan.xlsx
@@ -977,7 +977,7 @@
         </is>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="R6" s="6" t="n">
         <v>48</v>
@@ -1003,12 +1003,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Build 2 let</t>
+          <t>Build let (løb)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Wales</t>
+          <t>Gentofte→Wales 8.-12.</t>
         </is>
       </c>
       <c r="E7" s="2" t="n"/>
@@ -1036,17 +1036,17 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>Rejseuge — let cykel/løb, vedligehold.</t>
+          <t>Løbefokus — ingen cykel i Wales. Trail Z2 + vandring. Rejsedag ons 8.</t>
         </is>
       </c>
       <c r="Q7" s="6" t="n">
         <v>48</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>320</v>
+        <v>300</v>
       </c>
       <c r="T7" s="6" t="n"/>
       <c r="U7" s="6" t="inlineStr">
@@ -1066,12 +1066,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Build 3</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Mallorca</t>
+          <t>Gentofte→Mallorca 16.</t>
         </is>
       </c>
       <c r="E8" s="2" t="n"/>
@@ -1099,17 +1099,17 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>Stor cykel-uge #2.</t>
+          <t>Man-ons Gentofte (VO2 tir), tor-søn Mallorca ride-block. Rejsedag tor 16.</t>
         </is>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="S8" s="6" t="n">
-        <v>215</v>
+        <v>430</v>
       </c>
       <c r="T8" s="6" t="n"/>
       <c r="U8" s="6" t="inlineStr">
@@ -1129,12 +1129,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Recovery</t>
+          <t>Build+</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Mallorca→Gentofte</t>
+          <t>Mallorca→hjem 22.</t>
         </is>
       </c>
       <c r="E9" s="3" t="n"/>
@@ -1162,17 +1162,17 @@
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>Restitution + rejsedag hjem.</t>
+          <t>Store cykeldage man-tir. Hjem ons 22. Langtur 26 km lør — ladder start. TSB-gulv -35.</t>
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>430</v>
+        <v>480</v>
       </c>
       <c r="T9" s="6" t="n"/>
       <c r="U9" s="6" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Build 1</t>
+          <t>Recovery</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1225,17 +1225,17 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Musik i Gentofte i ugen efter (31/7–2/8) – planlæg let.</t>
+          <t>Fuld aflastning + FTP-test ons + threshold-test tor. Musik i Gentofte fre-søn.</t>
         </is>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="S10" s="6" t="n">
-        <v>380</v>
+        <v>200</v>
       </c>
       <c r="T10" s="6" t="n"/>
       <c r="U10" s="6" t="inlineStr">
@@ -1255,12 +1255,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Build 2</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Gentofte</t>
+          <t>Gentofte→fly søn 9.</t>
         </is>
       </c>
       <c r="E11" s="2" t="n"/>
@@ -1288,17 +1288,17 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>Svømme-fokus øges mod Christiansborg Rundt.</t>
+          <t>Langtur 28-30 km. OW-svøm starter tor. Fly Mallorca søn 9. aug.</t>
         </is>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>470</v>
+        <v>420</v>
       </c>
       <c r="T11" s="6" t="n"/>
       <c r="U11" s="6" t="inlineStr">
@@ -1318,12 +1318,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Build 3</t>
+          <t>Build+</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Mallorca</t>
+          <t>Mallorca (hjem 16.)</t>
         </is>
       </c>
       <c r="E12" s="2" t="n"/>
@@ -1351,14 +1351,14 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Sidste store blok før pre-race.</t>
+          <t>Camp #2. TSB-gulv -35 dagligt. Hjem søn 16. aug.</t>
         </is>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="S12" s="6" t="n">
         <v>500</v>
@@ -1381,12 +1381,12 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Pre-race</t>
+          <t>Taper</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Gentofte</t>
+          <t>Gentofte→Norge lør 22.</t>
         </is>
       </c>
       <c r="E13" s="4" t="n"/>
@@ -1414,17 +1414,17 @@
       </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>Svømme-specifik uge, nedtrapning starter. Norway 22–24/8 – planlæg rejse.</t>
+          <t>Sidste langtur 32 km TIRSDAG. OW-svøm x2. Norge lør 22.</t>
         </is>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>275</v>
+        <v>300</v>
       </c>
       <c r="T13" s="6" t="n"/>
       <c r="U13" s="6" t="inlineStr">
@@ -1444,12 +1444,12 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Race</t>
+          <t>Taper/RACE</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Christiansborg Rundt 29/8</t>
+          <t>Norge→hjem man 24.</t>
         </is>
       </c>
       <c r="E14" s="5" t="n"/>
@@ -1477,17 +1477,17 @@
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>Race week: 2000 m svøm 29/8. Taper ind, kort løb.</t>
+          <t>⭐ Christiansborg Rundt lør 29. aug. OW-tilvænning tir.</t>
         </is>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="S14" s="6" t="n">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="T14" s="6" t="n"/>
       <c r="U14" s="6" t="inlineStr">
@@ -1507,12 +1507,12 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Médoc</t>
+          <t>RACE</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Bordeaux – Marathon Médoc 5/9</t>
+          <t>Gentofte→Bordeaux tor</t>
         </is>
       </c>
       <c r="E15" s="5" t="n"/>
@@ -1540,17 +1540,17 @@
       </c>
       <c r="P15" s="5" t="inlineStr">
         <is>
-          <t>Marathon Médoc 5/9. Efter race: planen forlænges med recovery/2027-base – udfyldes når vi når hertil.</t>
+          <t>🏆 Marathon du Médoc lør 5. sep. Fly tor 3. sep.</t>
         </is>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="T15" s="6" t="n"/>
       <c r="U15" s="6" t="inlineStr">

</xml_diff>